<commit_message>
S2 Table: first 100 SICAPv2 result folders in folder order, without regard to Dice
H.A. clarified that the 100 reviewed SICAPv2 images are the first 100 result
folders as Drive lists them (0, 10, 11, 100, ...), not the first 100 with
Dice < 0.80. make_S2_table.py and the review text follow this rule: 4 slides of
3 patients, 23 in the official test partition, 76 with Dice < 0.80. Only the
PANDA cases are described as failure-selected.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PANDA_Reproducibility/supporting_information/S2_Table.xlsx
+++ b/PANDA_Reproducibility/supporting_information/S2_Table.xlsx
@@ -548,21 +548,21 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1000.jpg</t>
+          <t>11.jpg</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>16B0022608_Block_Region_0_5_24_xini_30647_yini_116942.jpg</t>
+          <t>16B0001851_Block_Region_1_2_1_xini_7827_yini_61834.jpg</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>16B0022608</t>
+          <t>16B0001851</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>296752</v>
+        <v>667360</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -574,7 +574,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -584,29 +584,29 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10001.jpg</t>
+          <t>100.jpg</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_10_14_xini_21274_yini_113891.jpg</t>
+          <t>16B0003388_Block_Region_13_7_1_xini_8636_yini_60797.jpg</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0003388</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>594051</v>
+        <v>325687</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>0.5668</v>
+        <v>0.8537</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -620,29 +620,29 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>10002.jpg</t>
+          <t>101.jpg</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_11_12_xini_19226_yini_114915.jpg</t>
+          <t>16B0003388_Block_Region_13_7_2_xini_9660_yini_60797.jpg</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0003388</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>594051</v>
+        <v>325687</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>0.589</v>
+        <v>0.9995000000000001</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -656,29 +656,29 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10004.jpg</t>
+          <t>102.jpg</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_11_14_xini_21274_yini_114915.jpg</t>
+          <t>16B0003388_Block_Region_13_7_3_xini_10684_yini_60797.jpg</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0003388</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>594051</v>
+        <v>325687</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>0.5768</v>
+        <v>0.8228</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -692,29 +692,29 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>10005.jpg</t>
+          <t>103.jpg</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_11_15_xini_22298_yini_114915.jpg</t>
+          <t>16B0003388_Block_Region_13_8_1_xini_8636_yini_61821.jpg</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0003388</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>594051</v>
+        <v>325687</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>0.5611</v>
+        <v>0.8774999999999999</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -728,29 +728,29 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>10006.jpg</t>
+          <t>104.jpg</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_12_12_xini_19226_yini_115939.jpg</t>
+          <t>16B0003388_Block_Region_13_8_2_xini_9660_yini_61821.jpg</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0003388</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>594051</v>
+        <v>325687</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>0.675</v>
+        <v>0.9224</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -764,29 +764,29 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>10007.jpg</t>
+          <t>105.jpg</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_12_13_xini_20250_yini_115939.jpg</t>
+          <t>16B0003388_Block_Region_13_8_3_xini_10684_yini_61821.jpg</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0003388</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>594051</v>
+        <v>325687</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>0.7609</v>
+        <v>0.8374</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -800,29 +800,29 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>10008.jpg</t>
+          <t>106.jpg</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_12_14_xini_21274_yini_115939.jpg</t>
+          <t>16B0003388_Block_Region_13_9_1_xini_8636_yini_62845.jpg</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0003388</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>594051</v>
+        <v>325687</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>0.7375</v>
+        <v>0.8459</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -836,29 +836,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10009.jpg</t>
+          <t>107.jpg</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_12_15_xini_22298_yini_115939.jpg</t>
+          <t>16B0003388_Block_Region_13_9_2_xini_9660_yini_62845.jpg</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0003388</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>594051</v>
+        <v>325687</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>0.6577</v>
+        <v>0.9941</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -872,33 +872,33 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1001.jpg</t>
+          <t>108.jpg</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16B0022608_Block_Region_0_5_25_xini_31671_yini_116942.jpg</t>
+          <t>16B0003388_Block_Region_13_9_3_xini_10684_yini_62845.jpg</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>16B0022608</t>
+          <t>16B0003388</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>296752</v>
+        <v>325687</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>0.8295</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -908,29 +908,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10010.jpg</t>
+          <t>109.jpg</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_13_13_xini_20250_yini_116963.jpg</t>
+          <t>16B0003388_Block_Region_5_10_0_xini_7339_yini_111140.jpg</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0003388</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>594051</v>
+        <v>325687</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>0.7581</v>
+        <v>0.8156</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -944,29 +944,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10012.jpg</t>
+          <t>110.jpg</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_13_15_xini_22298_yini_116963.jpg</t>
+          <t>16B0003388_Block_Region_5_10_1_xini_8363_yini_111140.jpg</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0003388</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>594051</v>
+        <v>325687</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>0.7308</v>
+        <v>0.9429</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -980,29 +980,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>10013.jpg</t>
+          <t>111.jpg</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_13_16_xini_23322_yini_116963.jpg</t>
+          <t>16B0003388_Block_Region_5_11_0_xini_7339_yini_112164.jpg</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0003388</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>594051</v>
+        <v>325687</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>0.5496</v>
+        <v>0.8912</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -1016,29 +1016,29 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>10014.jpg</t>
+          <t>112.jpg</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_14_13_xini_20250_yini_117987.jpg</t>
+          <t>16B0003388_Block_Region_5_11_1_xini_8363_yini_112164.jpg</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0003388</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>594051</v>
+        <v>325687</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>0.7229</v>
+        <v>0.9489</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -1052,29 +1052,29 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>10017.jpg</t>
+          <t>113.jpg</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_14_16_xini_23322_yini_117987.jpg</t>
+          <t>16B0003388_Block_Region_5_11_3_xini_10411_yini_112164.jpg</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0003388</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>594051</v>
+        <v>325687</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>0.539</v>
+        <v>0.9657</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -1088,29 +1088,29 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>10018.jpg</t>
+          <t>114.jpg</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_15_14_xini_21274_yini_119011.jpg</t>
+          <t>16B0003388_Block_Region_5_12_1_xini_8363_yini_113188.jpg</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0003388</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>594051</v>
+        <v>325687</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>0.66</v>
+        <v>0.9156</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -1124,29 +1124,29 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10019.jpg</t>
+          <t>115.jpg</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_15_15_xini_22298_yini_119011.jpg</t>
+          <t>16B0003388_Block_Region_5_13_1_xini_8363_yini_114212.jpg</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0003388</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>594051</v>
+        <v>325687</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>0.615</v>
+        <v>0.8362000000000001</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -1160,29 +1160,29 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>1002.jpg</t>
+          <t>116.jpg</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>16B0022608_Block_Region_0_5_7_xini_13239_yini_116942.jpg</t>
+          <t>16B0003388_Block_Region_5_13_2_xini_9387_yini_114212.jpg</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>16B0022608</t>
+          <t>16B0003388</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>296752</v>
+        <v>325687</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>0.3716</v>
+        <v>0.7717000000000001</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -1196,29 +1196,29 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>10020.jpg</t>
+          <t>117.jpg</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_15_16_xini_23322_yini_119011.jpg</t>
+          <t>16B0003388_Block_Region_5_14_2_xini_9387_yini_115236.jpg</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0003388</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>594051</v>
+        <v>325687</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>0.5121</v>
+        <v>0.6322</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -1232,29 +1232,29 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>10021.jpg</t>
+          <t>118.jpg</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_15_17_xini_24346_yini_119011.jpg</t>
+          <t>16B0003388_Block_Region_5_14_3_xini_10411_yini_115236.jpg</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0003388</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>594051</v>
+        <v>325687</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>0.5232</v>
+        <v>0.6166</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -1268,29 +1268,29 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>10022.jpg</t>
+          <t>119.jpg</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_16_14_xini_21274_yini_120035.jpg</t>
+          <t>16B0003388_Block_Region_5_14_4_xini_11435_yini_115236.jpg</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0003388</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>594051</v>
+        <v>325687</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>0</v>
+        <v>0.6492</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -1304,29 +1304,29 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>10023.jpg</t>
+          <t>120.jpg</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_16_15_xini_22298_yini_120035.jpg</t>
+          <t>16B0003388_Block_Region_5_15_2_xini_9387_yini_116260.jpg</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0003388</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>594051</v>
+        <v>325687</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>0.5994</v>
+        <v>0.5908</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -1340,29 +1340,29 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>10025.jpg</t>
+          <t>121.jpg</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_16_17_xini_24346_yini_120035.jpg</t>
+          <t>16B0003388_Block_Region_5_15_3_xini_10411_yini_116260.jpg</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0003388</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>594051</v>
+        <v>325687</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G26" t="n">
-        <v>0.5898</v>
+        <v>0.7883</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -1376,29 +1376,29 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>10026.jpg</t>
+          <t>122.jpg</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_17_15_xini_22298_yini_121059.jpg</t>
+          <t>16B0003388_Block_Region_5_15_4_xini_11435_yini_116260.jpg</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0003388</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>594051</v>
+        <v>325687</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>0.6239</v>
+        <v>0.9592000000000001</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
@@ -1412,21 +1412,21 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>10027.jpg</t>
+          <t>1000.jpg</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_17_16_xini_23322_yini_121059.jpg</t>
+          <t>16B0022608_Block_Region_0_5_24_xini_30647_yini_116942.jpg</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1434,11 +1434,11 @@
         </is>
       </c>
       <c r="G28" t="n">
-        <v>0.6177</v>
+        <v>0</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1448,21 +1448,21 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>10028.jpg</t>
+          <t>1001.jpg</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_17_17_xini_24346_yini_121059.jpg</t>
+          <t>16B0022608_Block_Region_0_5_25_xini_31671_yini_116942.jpg</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1470,11 +1470,11 @@
         </is>
       </c>
       <c r="G29" t="n">
-        <v>0.5995</v>
+        <v>0</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1484,21 +1484,21 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>10029.jpg</t>
+          <t>1002.jpg</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_1_0_xini_6938_yini_104675.jpg</t>
+          <t>16B0022608_Block_Region_0_5_7_xini_13239_yini_116942.jpg</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1506,11 +1506,11 @@
         </is>
       </c>
       <c r="G30" t="n">
-        <v>0</v>
+        <v>0.3716</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1556,21 +1556,21 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>10030.jpg</t>
+          <t>1004.jpg</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_1_1_xini_7962_yini_104675.jpg</t>
+          <t>16B0022608_Block_Region_0_5_9_xini_15287_yini_116942.jpg</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1578,11 +1578,11 @@
         </is>
       </c>
       <c r="G32" t="n">
-        <v>0</v>
+        <v>0.5804</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1592,21 +1592,21 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>10031.jpg</t>
+          <t>1005.jpg</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_1_2_xini_8986_yini_104675.jpg</t>
+          <t>16B0022608_Block_Region_0_6_12_xini_18359_yini_117966.jpg</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -1614,11 +1614,11 @@
         </is>
       </c>
       <c r="G33" t="n">
-        <v>0</v>
+        <v>0.3284</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1628,21 +1628,21 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>10032.jpg</t>
+          <t>1006.jpg</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_1_3_xini_10010_yini_104675.jpg</t>
+          <t>16B0022608_Block_Region_0_6_17_xini_23479_yini_117966.jpg</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -1664,21 +1664,21 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>10033.jpg</t>
+          <t>1007.jpg</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_1_4_xini_11034_yini_104675.jpg</t>
+          <t>16B0022608_Block_Region_0_6_18_xini_24503_yini_117966.jpg</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -1686,11 +1686,11 @@
         </is>
       </c>
       <c r="G35" t="n">
-        <v>0.2644</v>
+        <v>0</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1700,21 +1700,21 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>10034.jpg</t>
+          <t>1008.jpg</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_1_5_xini_12058_yini_104675.jpg</t>
+          <t>16B0022608_Block_Region_0_6_19_xini_25527_yini_117966.jpg</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -1722,11 +1722,11 @@
         </is>
       </c>
       <c r="G36" t="n">
-        <v>0.4908</v>
+        <v>0</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1736,21 +1736,21 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>10035.jpg</t>
+          <t>1009.jpg</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_1_6_xini_13082_yini_104675.jpg</t>
+          <t>16B0022608_Block_Region_0_6_20_xini_26551_yini_117966.jpg</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -1758,11 +1758,11 @@
         </is>
       </c>
       <c r="G37" t="n">
-        <v>0.6062</v>
+        <v>0</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1772,21 +1772,21 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>10036.jpg</t>
+          <t>1010.jpg</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_1_7_xini_14106_yini_104675.jpg</t>
+          <t>16B0022608_Block_Region_0_6_21_xini_27575_yini_117966.jpg</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -1794,11 +1794,11 @@
         </is>
       </c>
       <c r="G38" t="n">
-        <v>0.5857</v>
+        <v>0</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1808,21 +1808,21 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>10037.jpg</t>
+          <t>1011.jpg</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_1_8_xini_15130_yini_104675.jpg</t>
+          <t>16B0022608_Block_Region_0_6_22_xini_28599_yini_117966.jpg</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -1830,11 +1830,11 @@
         </is>
       </c>
       <c r="G39" t="n">
-        <v>0.5402</v>
+        <v>0</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1844,21 +1844,21 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>10038.jpg</t>
+          <t>1012.jpg</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_2_1_xini_7962_yini_105699.jpg</t>
+          <t>16B0022608_Block_Region_0_6_23_xini_29623_yini_117966.jpg</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
@@ -1880,21 +1880,21 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>10039.jpg</t>
+          <t>1013.jpg</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_2_2_xini_8986_yini_105699.jpg</t>
+          <t>16B0022608_Block_Region_0_6_24_xini_30647_yini_117966.jpg</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
@@ -1916,12 +1916,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>1004.jpg</t>
+          <t>1014.jpg</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>16B0022608_Block_Region_0_5_9_xini_15287_yini_116942.jpg</t>
+          <t>16B0022608_Block_Region_0_6_25_xini_31671_yini_117966.jpg</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1938,11 +1938,11 @@
         </is>
       </c>
       <c r="G42" t="n">
-        <v>0.5804</v>
+        <v>0</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1952,21 +1952,21 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>10040.jpg</t>
+          <t>1015.jpg</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_2_3_xini_10010_yini_105699.jpg</t>
+          <t>16B0022608_Block_Region_2_0_0_xini_6703_yini_60132.jpg</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
@@ -1974,11 +1974,11 @@
         </is>
       </c>
       <c r="G43" t="n">
-        <v>0</v>
+        <v>0.0232</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1988,21 +1988,21 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>10041.jpg</t>
+          <t>1016.jpg</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_2_6_xini_13082_yini_105699.jpg</t>
+          <t>16B0022608_Block_Region_2_0_1_xini_7727_yini_60132.jpg</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -2010,7 +2010,7 @@
         </is>
       </c>
       <c r="G44" t="n">
-        <v>0.5449000000000001</v>
+        <v>0.147</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
@@ -2024,21 +2024,21 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>10043.jpg</t>
+          <t>1017.jpg</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_2_8_xini_15130_yini_105699.jpg</t>
+          <t>16B0022608_Block_Region_2_1_0_xini_6703_yini_61156.jpg</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -2046,7 +2046,7 @@
         </is>
       </c>
       <c r="G45" t="n">
-        <v>0.5886</v>
+        <v>0.4221</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
@@ -2060,21 +2060,21 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>10044.jpg</t>
+          <t>1018.jpg</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_2_9_xini_16154_yini_105699.jpg</t>
+          <t>16B0022608_Block_Region_2_1_1_xini_7727_yini_61156.jpg</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
@@ -2082,7 +2082,7 @@
         </is>
       </c>
       <c r="G46" t="n">
-        <v>0.6444</v>
+        <v>0.5966</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
@@ -2096,21 +2096,21 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>10045.jpg</t>
+          <t>1019.jpg</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_3_10_xini_17178_yini_106723.jpg</t>
+          <t>16B0022608_Block_Region_2_1_2_xini_8751_yini_61156.jpg</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -2118,7 +2118,7 @@
         </is>
       </c>
       <c r="G47" t="n">
-        <v>0.7095</v>
+        <v>0.3887</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
@@ -2132,21 +2132,21 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>10046.jpg</t>
+          <t>1020.jpg</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_3_7_xini_14106_yini_106723.jpg</t>
+          <t>16B0022608_Block_Region_2_1_3_xini_9775_yini_61156.jpg</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -2154,7 +2154,7 @@
         </is>
       </c>
       <c r="G48" t="n">
-        <v>0.6195000000000001</v>
+        <v>0.1494</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
@@ -2168,21 +2168,21 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>10048.jpg</t>
+          <t>1021.jpg</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_3_9_xini_16154_yini_106723.jpg</t>
+          <t>16B0022608_Block_Region_2_2_1_xini_7727_yini_62180.jpg</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
         </is>
       </c>
       <c r="G49" t="n">
-        <v>0.6556999999999999</v>
+        <v>0.6172</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
@@ -2204,21 +2204,21 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>10049.jpg</t>
+          <t>1022.jpg</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_4_10_xini_17178_yini_107747.jpg</t>
+          <t>16B0022608_Block_Region_2_2_2_xini_8751_yini_62180.jpg</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E50" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
@@ -2226,7 +2226,7 @@
         </is>
       </c>
       <c r="G50" t="n">
-        <v>0.7251</v>
+        <v>0.4414</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
@@ -2240,12 +2240,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>1005.jpg</t>
+          <t>1023.jpg</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>16B0022608_Block_Region_0_6_12_xini_18359_yini_117966.jpg</t>
+          <t>16B0022608_Block_Region_2_2_3_xini_9775_yini_62180.jpg</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2262,7 +2262,7 @@
         </is>
       </c>
       <c r="G51" t="n">
-        <v>0.3284</v>
+        <v>0.1139</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
@@ -2276,21 +2276,21 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>10050.jpg</t>
+          <t>1024.jpg</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_4_7_xini_14106_yini_107747.jpg</t>
+          <t>16B0022608_Block_Region_2_2_4_xini_10799_yini_62180.jpg</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -2298,7 +2298,7 @@
         </is>
       </c>
       <c r="G52" t="n">
-        <v>0.6511</v>
+        <v>0.339</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
@@ -2312,21 +2312,21 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>10053.jpg</t>
+          <t>1025.jpg</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_5_10_xini_17178_yini_108771.jpg</t>
+          <t>16B0022608_Block_Region_2_3_2_xini_8751_yini_63204.jpg</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E53" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
@@ -2334,7 +2334,7 @@
         </is>
       </c>
       <c r="G53" t="n">
-        <v>0.7187</v>
+        <v>0</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
@@ -2348,21 +2348,21 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>10054.jpg</t>
+          <t>1026.jpg</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_5_11_xini_18202_yini_108771.jpg</t>
+          <t>16B0022608_Block_Region_2_3_3_xini_9775_yini_63204.jpg</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E54" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -2370,7 +2370,7 @@
         </is>
       </c>
       <c r="G54" t="n">
-        <v>0.6912</v>
+        <v>0.2027</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
@@ -2384,21 +2384,21 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>10055.jpg</t>
+          <t>1027.jpg</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_5_8_xini_15130_yini_108771.jpg</t>
+          <t>16B0022608_Block_Region_2_3_4_xini_10799_yini_63204.jpg</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E55" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
@@ -2406,7 +2406,7 @@
         </is>
       </c>
       <c r="G55" t="n">
-        <v>0.632</v>
+        <v>0.2875</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
@@ -2420,21 +2420,21 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>10057.jpg</t>
+          <t>1028.jpg</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_6_10_xini_17178_yini_109795.jpg</t>
+          <t>16B0022608_Block_Region_2_3_5_xini_11823_yini_63204.jpg</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
         </is>
       </c>
       <c r="G56" t="n">
-        <v>0.6936</v>
+        <v>0.3532</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
@@ -2456,21 +2456,21 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>10058.jpg</t>
+          <t>1029.jpg</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_6_11_xini_18202_yini_109795.jpg</t>
+          <t>16B0022608_Block_Region_2_3_6_xini_12847_yini_63204.jpg</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E57" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
@@ -2478,11 +2478,11 @@
         </is>
       </c>
       <c r="G57" t="n">
-        <v>0.6802</v>
+        <v>0</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2492,21 +2492,21 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>10059.jpg</t>
+          <t>1030.jpg</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_6_8_xini_15130_yini_109795.jpg</t>
+          <t>16B0022608_Block_Region_2_3_7_xini_13871_yini_63204.jpg</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E58" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
@@ -2514,11 +2514,11 @@
         </is>
       </c>
       <c r="G58" t="n">
-        <v>0.5863</v>
+        <v>0</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2528,12 +2528,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>1006.jpg</t>
+          <t>1031.jpg</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>16B0022608_Block_Region_0_6_17_xini_23479_yini_117966.jpg</t>
+          <t>16B0022608_Block_Region_2_4_10_xini_16943_yini_64228.jpg</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2564,21 +2564,21 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>10060.jpg</t>
+          <t>1032.jpg</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_6_9_xini_16154_yini_109795.jpg</t>
+          <t>16B0022608_Block_Region_2_4_11_xini_17967_yini_64228.jpg</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E60" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
@@ -2586,11 +2586,11 @@
         </is>
       </c>
       <c r="G60" t="n">
-        <v>0.662</v>
+        <v>0</v>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2600,21 +2600,21 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>10061.jpg</t>
+          <t>1033.jpg</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_7_10_xini_17178_yini_110819.jpg</t>
+          <t>16B0022608_Block_Region_2_4_3_xini_9775_yini_64228.jpg</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
@@ -2622,7 +2622,7 @@
         </is>
       </c>
       <c r="G61" t="n">
-        <v>0.6662</v>
+        <v>0</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
@@ -2636,21 +2636,21 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>10062.jpg</t>
+          <t>1034.jpg</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_7_11_xini_18202_yini_110819.jpg</t>
+          <t>16B0022608_Block_Region_2_4_4_xini_10799_yini_64228.jpg</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E62" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
@@ -2658,7 +2658,7 @@
         </is>
       </c>
       <c r="G62" t="n">
-        <v>0.6656</v>
+        <v>0.484</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
@@ -2672,21 +2672,21 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>10063.jpg</t>
+          <t>1035.jpg</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_7_12_xini_19226_yini_110819.jpg</t>
+          <t>16B0022608_Block_Region_2_4_5_xini_11823_yini_64228.jpg</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E63" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
         </is>
       </c>
       <c r="G63" t="n">
-        <v>0.7364000000000001</v>
+        <v>0.2256</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
@@ -2708,21 +2708,21 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>10064.jpg</t>
+          <t>1036.jpg</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_7_9_xini_16154_yini_110819.jpg</t>
+          <t>16B0022608_Block_Region_2_4_6_xini_12847_yini_64228.jpg</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E64" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
@@ -2730,11 +2730,11 @@
         </is>
       </c>
       <c r="G64" t="n">
-        <v>0.6715</v>
+        <v>0</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2744,21 +2744,21 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>10065.jpg</t>
+          <t>1037.jpg</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_8_10_xini_17178_yini_111843.jpg</t>
+          <t>16B0022608_Block_Region_2_4_7_xini_13871_yini_64228.jpg</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E65" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
@@ -2766,11 +2766,11 @@
         </is>
       </c>
       <c r="G65" t="n">
-        <v>0.6441</v>
+        <v>0</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2780,21 +2780,21 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>10066.jpg</t>
+          <t>1038.jpg</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_8_11_xini_18202_yini_111843.jpg</t>
+          <t>16B0022608_Block_Region_2_4_8_xini_14895_yini_64228.jpg</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E66" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
@@ -2802,11 +2802,11 @@
         </is>
       </c>
       <c r="G66" t="n">
-        <v>0.656</v>
+        <v>0</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2816,21 +2816,21 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>10067.jpg</t>
+          <t>1039.jpg</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_8_12_xini_19226_yini_111843.jpg</t>
+          <t>16B0022608_Block_Region_2_4_9_xini_15919_yini_64228.jpg</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022608</t>
         </is>
       </c>
       <c r="E67" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
@@ -2838,11 +2838,11 @@
         </is>
       </c>
       <c r="G67" t="n">
-        <v>0.6933</v>
+        <v>0</v>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2852,21 +2852,21 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>10068.jpg</t>
+          <t>1040.jpg</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_8_13_xini_20250_yini_111843.jpg</t>
+          <t>16B0022610_Block_Region_10_0_0_xini_31766_yini_3272.jpg</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E68" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
@@ -2874,7 +2874,7 @@
         </is>
       </c>
       <c r="G68" t="n">
-        <v>0.738</v>
+        <v>0.2955</v>
       </c>
       <c r="H68" t="inlineStr">
         <is>
@@ -2888,21 +2888,21 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>10069.jpg</t>
+          <t>1041.jpg</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_9_11_xini_18202_yini_112867.jpg</t>
+          <t>16B0022610_Block_Region_10_0_1_xini_32790_yini_3272.jpg</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E69" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
@@ -2910,7 +2910,7 @@
         </is>
       </c>
       <c r="G69" t="n">
-        <v>0.5435</v>
+        <v>0.7096</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
@@ -2924,17 +2924,17 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>1007.jpg</t>
+          <t>1042.jpg</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>16B0022608_Block_Region_0_6_18_xini_24503_yini_117966.jpg</t>
+          <t>16B0022610_Block_Region_10_0_2_xini_33814_yini_3272.jpg</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>16B0022608</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E70" t="n">
@@ -2946,11 +2946,11 @@
         </is>
       </c>
       <c r="G70" t="n">
-        <v>0</v>
+        <v>0.8627</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2960,21 +2960,21 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>10070.jpg</t>
+          <t>1043.jpg</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_9_12_xini_19226_yini_112867.jpg</t>
+          <t>16B0022610_Block_Region_10_0_3_xini_34838_yini_3272.jpg</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E71" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
@@ -2982,7 +2982,7 @@
         </is>
       </c>
       <c r="G71" t="n">
-        <v>0.6689000000000001</v>
+        <v>0.9256</v>
       </c>
       <c r="H71" t="inlineStr">
         <is>
@@ -2996,21 +2996,21 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>10071.jpg</t>
+          <t>1044.jpg</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_9_13_xini_20250_yini_112867.jpg</t>
+          <t>16B0022610_Block_Region_10_0_4_xini_35862_yini_3272.jpg</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E72" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F72" t="inlineStr">
         <is>
@@ -3018,7 +3018,7 @@
         </is>
       </c>
       <c r="G72" t="n">
-        <v>0.6958</v>
+        <v>0.7445000000000001</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
@@ -3032,21 +3032,21 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>10072.jpg</t>
+          <t>1045.jpg</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>17B0031877_Block_Region_4_9_14_xini_21274_yini_112867.jpg</t>
+          <t>16B0022610_Block_Region_10_0_5_xini_36886_yini_3272.jpg</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>17B0031877</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E73" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
@@ -3054,7 +3054,7 @@
         </is>
       </c>
       <c r="G73" t="n">
-        <v>0.6317</v>
+        <v>0.6446</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
@@ -3068,21 +3068,21 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>10073.jpg</t>
+          <t>1046.jpg</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>17B0031879_Block_Region_0_0_10_xini_20803_yini_119794.jpg</t>
+          <t>16B0022610_Block_Region_10_0_6_xini_37910_yini_3272.jpg</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>17B0031879</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E74" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
@@ -3090,11 +3090,11 @@
         </is>
       </c>
       <c r="G74" t="n">
-        <v>0</v>
+        <v>0.7116</v>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3104,21 +3104,21 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>10074.jpg</t>
+          <t>1047.jpg</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>17B0031879_Block_Region_0_0_11_xini_21827_yini_119794.jpg</t>
+          <t>16B0022610_Block_Region_10_0_7_xini_38934_yini_3272.jpg</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>17B0031879</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E75" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
@@ -3140,21 +3140,21 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>10075.jpg</t>
+          <t>1048.jpg</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>17B0031879_Block_Region_0_0_12_xini_22851_yini_119794.jpg</t>
+          <t>16B0022610_Block_Region_10_1_0_xini_31766_yini_4296.jpg</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>17B0031879</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E76" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
@@ -3162,11 +3162,11 @@
         </is>
       </c>
       <c r="G76" t="n">
-        <v>0</v>
+        <v>0.5617</v>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3176,21 +3176,21 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>10076.jpg</t>
+          <t>1049.jpg</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>17B0031879_Block_Region_0_10_3_xini_13635_yini_130034.jpg</t>
+          <t>16B0022610_Block_Region_10_1_1_xini_32790_yini_4296.jpg</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>17B0031879</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E77" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
         </is>
       </c>
       <c r="G77" t="n">
-        <v>0</v>
+        <v>0.7879</v>
       </c>
       <c r="H77" t="inlineStr">
         <is>
@@ -3212,21 +3212,21 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>10077.jpg</t>
+          <t>1050.jpg</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>17B0031879_Block_Region_0_10_4_xini_14659_yini_130034.jpg</t>
+          <t>16B0022610_Block_Region_10_1_2_xini_33814_yini_4296.jpg</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>17B0031879</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E78" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F78" t="inlineStr">
         <is>
@@ -3234,7 +3234,7 @@
         </is>
       </c>
       <c r="G78" t="n">
-        <v>0.7459</v>
+        <v>0.8607</v>
       </c>
       <c r="H78" t="inlineStr">
         <is>
@@ -3248,21 +3248,21 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>10079.jpg</t>
+          <t>1051.jpg</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>17B0031879_Block_Region_0_10_6_xini_16707_yini_130034.jpg</t>
+          <t>16B0022610_Block_Region_10_1_3_xini_34838_yini_4296.jpg</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>17B0031879</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E79" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
@@ -3270,7 +3270,7 @@
         </is>
       </c>
       <c r="G79" t="n">
-        <v>0.748</v>
+        <v>0.9159</v>
       </c>
       <c r="H79" t="inlineStr">
         <is>
@@ -3284,17 +3284,17 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>1008.jpg</t>
+          <t>1052.jpg</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>16B0022608_Block_Region_0_6_19_xini_25527_yini_117966.jpg</t>
+          <t>16B0022610_Block_Region_10_1_4_xini_35862_yini_4296.jpg</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>16B0022608</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E80" t="n">
@@ -3306,11 +3306,11 @@
         </is>
       </c>
       <c r="G80" t="n">
-        <v>0</v>
+        <v>0.8090000000000001</v>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3320,21 +3320,21 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>10080.jpg</t>
+          <t>1053.jpg</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>17B0031879_Block_Region_0_11_2_xini_12611_yini_131058.jpg</t>
+          <t>16B0022610_Block_Region_10_1_5_xini_36886_yini_4296.jpg</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>17B0031879</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E81" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F81" t="inlineStr">
         <is>
@@ -3342,7 +3342,7 @@
         </is>
       </c>
       <c r="G81" t="n">
-        <v>0.7399</v>
+        <v>0.5699</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
@@ -3356,21 +3356,21 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>10081.jpg</t>
+          <t>1054.jpg</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>17B0031879_Block_Region_0_11_3_xini_13635_yini_131058.jpg</t>
+          <t>16B0022610_Block_Region_10_1_6_xini_37910_yini_4296.jpg</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>17B0031879</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E82" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F82" t="inlineStr">
         <is>
@@ -3378,7 +3378,7 @@
         </is>
       </c>
       <c r="G82" t="n">
-        <v>0.7572</v>
+        <v>0.6946</v>
       </c>
       <c r="H82" t="inlineStr">
         <is>
@@ -3392,21 +3392,21 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>10082.jpg</t>
+          <t>1055.jpg</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>17B0031879_Block_Region_0_11_4_xini_14659_yini_131058.jpg</t>
+          <t>16B0022610_Block_Region_10_1_7_xini_38934_yini_4296.jpg</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>17B0031879</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E83" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F83" t="inlineStr">
         <is>
@@ -3414,7 +3414,7 @@
         </is>
       </c>
       <c r="G83" t="n">
-        <v>0.781</v>
+        <v>0</v>
       </c>
       <c r="H83" t="inlineStr">
         <is>
@@ -3428,21 +3428,21 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>10083.jpg</t>
+          <t>1056.jpg</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>17B0031879_Block_Region_0_11_5_xini_15683_yini_131058.jpg</t>
+          <t>16B0022610_Block_Region_10_2_4_xini_35862_yini_5320.jpg</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>17B0031879</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E84" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
@@ -3450,7 +3450,7 @@
         </is>
       </c>
       <c r="G84" t="n">
-        <v>0.7519</v>
+        <v>0.7859</v>
       </c>
       <c r="H84" t="inlineStr">
         <is>
@@ -3464,21 +3464,21 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>10084.jpg</t>
+          <t>1057.jpg</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>17B0031879_Block_Region_0_12_2_xini_12611_yini_132082.jpg</t>
+          <t>16B0022610_Block_Region_10_2_5_xini_36886_yini_5320.jpg</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>17B0031879</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E85" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F85" t="inlineStr">
         <is>
@@ -3486,7 +3486,7 @@
         </is>
       </c>
       <c r="G85" t="n">
-        <v>0.707</v>
+        <v>0.7752</v>
       </c>
       <c r="H85" t="inlineStr">
         <is>
@@ -3500,21 +3500,21 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>10086.jpg</t>
+          <t>1058.jpg</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>17B0031879_Block_Region_0_12_4_xini_14659_yini_132082.jpg</t>
+          <t>16B0022610_Block_Region_10_2_6_xini_37910_yini_5320.jpg</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>17B0031879</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E86" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F86" t="inlineStr">
         <is>
@@ -3522,7 +3522,7 @@
         </is>
       </c>
       <c r="G86" t="n">
-        <v>0.5523</v>
+        <v>0.7993</v>
       </c>
       <c r="H86" t="inlineStr">
         <is>
@@ -3536,21 +3536,21 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>10087.jpg</t>
+          <t>1059.jpg</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>17B0031879_Block_Region_0_12_5_xini_15683_yini_132082.jpg</t>
+          <t>16B0022610_Block_Region_10_2_7_xini_38934_yini_5320.jpg</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>17B0031879</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E87" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F87" t="inlineStr">
         <is>
@@ -3572,21 +3572,21 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>10088.jpg</t>
+          <t>1060.jpg</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>17B0031879_Block_Region_0_13_2_xini_12611_yini_133106.jpg</t>
+          <t>16B0022610_Block_Region_9_0_16_xini_27702_yini_5958.jpg</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>17B0031879</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E88" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F88" t="inlineStr">
         <is>
@@ -3594,7 +3594,7 @@
         </is>
       </c>
       <c r="G88" t="n">
-        <v>0.186</v>
+        <v>0.7792</v>
       </c>
       <c r="H88" t="inlineStr">
         <is>
@@ -3608,21 +3608,21 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>10089.jpg</t>
+          <t>1061.jpg</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>17B0031879_Block_Region_0_13_3_xini_13635_yini_133106.jpg</t>
+          <t>16B0022610_Block_Region_9_0_17_xini_28726_yini_5958.jpg</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>17B0031879</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E89" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F89" t="inlineStr">
         <is>
@@ -3630,11 +3630,11 @@
         </is>
       </c>
       <c r="G89" t="n">
-        <v>0</v>
+        <v>0.8243</v>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3644,17 +3644,17 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>1009.jpg</t>
+          <t>1062.jpg</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>16B0022608_Block_Region_0_6_20_xini_26551_yini_117966.jpg</t>
+          <t>16B0022610_Block_Region_9_0_18_xini_29750_yini_5958.jpg</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>16B0022608</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E90" t="n">
@@ -3666,11 +3666,11 @@
         </is>
       </c>
       <c r="G90" t="n">
-        <v>0</v>
+        <v>0.8851</v>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3680,21 +3680,21 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>10090.jpg</t>
+          <t>1063.jpg</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>17B0031879_Block_Region_0_13_4_xini_14659_yini_133106.jpg</t>
+          <t>16B0022610_Block_Region_9_0_19_xini_30774_yini_5958.jpg</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>17B0031879</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E91" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F91" t="inlineStr">
         <is>
@@ -3702,7 +3702,7 @@
         </is>
       </c>
       <c r="G91" t="n">
-        <v>0</v>
+        <v>0.6296</v>
       </c>
       <c r="H91" t="inlineStr">
         <is>
@@ -3716,21 +3716,21 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>10091.jpg</t>
+          <t>1064.jpg</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>17B0031879_Block_Region_0_14_1_xini_11587_yini_134130.jpg</t>
+          <t>16B0022610_Block_Region_9_10_2_xini_13366_yini_16198.jpg</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>17B0031879</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E92" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
@@ -3752,21 +3752,21 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>10092.jpg</t>
+          <t>1065.jpg</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>17B0031879_Block_Region_0_14_2_xini_12611_yini_134130.jpg</t>
+          <t>16B0022610_Block_Region_9_10_3_xini_14390_yini_16198.jpg</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>17B0031879</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E93" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F93" t="inlineStr">
         <is>
@@ -3788,21 +3788,21 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>10093.jpg</t>
+          <t>1066.jpg</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>17B0031879_Block_Region_0_14_3_xini_13635_yini_134130.jpg</t>
+          <t>16B0022610_Block_Region_9_10_4_xini_15414_yini_16198.jpg</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>17B0031879</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E94" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
@@ -3824,21 +3824,21 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>10094.jpg</t>
+          <t>1067.jpg</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>17B0031879_Block_Region_0_14_4_xini_14659_yini_134130.jpg</t>
+          <t>16B0022610_Block_Region_9_10_5_xini_16438_yini_16198.jpg</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>17B0031879</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E95" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F95" t="inlineStr">
         <is>
@@ -3860,21 +3860,21 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>10095.jpg</t>
+          <t>1068.jpg</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>17B0031879_Block_Region_0_15_1_xini_11587_yini_135154.jpg</t>
+          <t>16B0022610_Block_Region_9_10_6_xini_17462_yini_16198.jpg</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>17B0031879</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E96" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F96" t="inlineStr">
         <is>
@@ -3896,21 +3896,21 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>10096.jpg</t>
+          <t>1069.jpg</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>17B0031879_Block_Region_0_15_2_xini_12611_yini_135154.jpg</t>
+          <t>16B0022610_Block_Region_9_11_2_xini_13366_yini_17222.jpg</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>17B0031879</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E97" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
@@ -3932,21 +3932,21 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>10097.jpg</t>
+          <t>1070.jpg</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>17B0031879_Block_Region_0_15_3_xini_13635_yini_135154.jpg</t>
+          <t>16B0022610_Block_Region_9_11_3_xini_14390_yini_17222.jpg</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>17B0031879</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E98" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F98" t="inlineStr">
         <is>
@@ -3968,21 +3968,21 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>10098.jpg</t>
+          <t>1071.jpg</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>17B0031879_Block_Region_0_15_4_xini_14659_yini_135154.jpg</t>
+          <t>16B0022610_Block_Region_9_11_4_xini_15414_yini_17222.jpg</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>17B0031879</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E99" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F99" t="inlineStr">
         <is>
@@ -4004,21 +4004,21 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>10099.jpg</t>
+          <t>1072.jpg</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>17B0031879_Block_Region_0_16_1_xini_11587_yini_136178.jpg</t>
+          <t>16B0022610_Block_Region_9_12_1_xini_12342_yini_18246.jpg</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>17B0031879</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E100" t="n">
-        <v>594051</v>
+        <v>296752</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
@@ -4040,17 +4040,17 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>1010.jpg</t>
+          <t>1073.jpg</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>16B0022608_Block_Region_0_6_21_xini_27575_yini_117966.jpg</t>
+          <t>16B0022610_Block_Region_9_12_2_xini_13366_yini_18246.jpg</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>16B0022608</t>
+          <t>16B0022610</t>
         </is>
       </c>
       <c r="E101" t="n">

</xml_diff>